<commit_message>
Add payment and registration downloads
</commit_message>
<xml_diff>
--- a/data/payments.xlsx
+++ b/data/payments.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="60">
   <si>
     <t>referenceId</t>
   </si>
@@ -167,6 +167,30 @@
   </si>
   <si>
     <t>2026-10-05T12:15:59.412Z</t>
+  </si>
+  <si>
+    <t>REG-20261007-3563S</t>
+  </si>
+  <si>
+    <t>SEMINAR</t>
+  </si>
+  <si>
+    <t>SELVAMUTHU GV</t>
+  </si>
+  <si>
+    <t>selvamuthugv@gmail.com</t>
+  </si>
+  <si>
+    <t>9985214722</t>
+  </si>
+  <si>
+    <t>eee</t>
+  </si>
+  <si>
+    <t>741852963sdfghj52</t>
+  </si>
+  <si>
+    <t>2026-10-07T05:34:20.743Z</t>
   </si>
 </sst>
 </file>
@@ -543,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -779,6 +803,53 @@
       </c>
       <c r="O5" t="s">
         <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6">
+        <v>250</v>
+      </c>
+      <c r="K6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>59</v>
+      </c>
+      <c r="N6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>